<commit_message>
Aus GP FP2 penalties
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1992" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1287ADBB-6F3C-4A38-9639-EDD5BAA7DDAC}"/>
+  <xr:revisionPtr revIDLastSave="2028" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96826851-0233-461D-A805-6804E36EDE61}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="2" r:id="rId1"/>
@@ -19,13 +19,14 @@
     <sheet name="2023" sheetId="5" r:id="rId4"/>
     <sheet name="2024" sheetId="6" r:id="rId5"/>
     <sheet name="2025" sheetId="7" r:id="rId6"/>
+    <sheet name="2026" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10387" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10428" uniqueCount="502">
   <si>
     <t>Year</t>
   </si>
@@ -1519,6 +1520,18 @@
   </si>
   <si>
     <t>Overturned</t>
+  </si>
+  <si>
+    <t>FP2</t>
+  </si>
+  <si>
+    <t>Performed practice start outside designated practice area</t>
+  </si>
+  <si>
+    <t>Nish Shetty, Pedro Lamy, Mathieu Remmerie, Matthew Selley</t>
+  </si>
+  <si>
+    <t>Car having mechanical problems</t>
   </si>
 </sst>
 </file>
@@ -1603,6 +1616,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -45655,4 +45672,166 @@
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
+  <dimension ref="A1:P4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="11" max="11" width="22.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2026</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>169</v>
+      </c>
+      <c r="D2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" t="s">
+        <v>498</v>
+      </c>
+      <c r="G2" t="s">
+        <v>125</v>
+      </c>
+      <c r="J2" t="s">
+        <v>91</v>
+      </c>
+      <c r="O2" t="s">
+        <v>499</v>
+      </c>
+      <c r="P2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2026</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
+        <v>498</v>
+      </c>
+      <c r="G3" t="s">
+        <v>274</v>
+      </c>
+      <c r="I3" t="s">
+        <v>331</v>
+      </c>
+      <c r="J3" t="s">
+        <v>84</v>
+      </c>
+      <c r="P3" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2026</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E4" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" t="s">
+        <v>498</v>
+      </c>
+      <c r="G4" t="s">
+        <v>278</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" t="s">
+        <v>285</v>
+      </c>
+      <c r="O4" t="s">
+        <v>501</v>
+      </c>
+      <c r="P4" t="s">
+        <v>500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
China FP1 & SQ
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2111" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48DBA661-180D-4FE8-89CC-F54C65640100}"/>
+  <xr:revisionPtr revIDLastSave="2139" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC7BEFB0-1BC9-4371-A697-4B59346C432C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10503" uniqueCount="514">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10521" uniqueCount="516">
   <si>
     <t>Year</t>
   </si>
@@ -1522,9 +1522,6 @@
     <t>Overturned</t>
   </si>
   <si>
-    <t>FP2</t>
-  </si>
-  <si>
     <t>Performed practice start outside designated practice area</t>
   </si>
   <si>
@@ -1568,6 +1565,15 @@
   </si>
   <si>
     <t>Cadillac</t>
+  </si>
+  <si>
+    <t>Performed practice start on the grid while another driver was stationary on the same side of the grid</t>
+  </si>
+  <si>
+    <t>Nish Shetty, Matthew Selley, Pedro Lamy, Zheng Honghai</t>
+  </si>
+  <si>
+    <t>Norris not on a push lap</t>
   </si>
 </sst>
 </file>
@@ -1652,6 +1658,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -45708,7 +45718,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -45784,7 +45794,7 @@
         <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>498</v>
+        <v>50</v>
       </c>
       <c r="G2" t="s">
         <v>125</v>
@@ -45793,10 +45803,10 @@
         <v>91</v>
       </c>
       <c r="O2" t="s">
+        <v>498</v>
+      </c>
+      <c r="P2" t="s">
         <v>499</v>
-      </c>
-      <c r="P2" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
@@ -45816,7 +45826,7 @@
         <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>498</v>
+        <v>50</v>
       </c>
       <c r="G3" t="s">
         <v>274</v>
@@ -45828,10 +45838,10 @@
         <v>84</v>
       </c>
       <c r="O3" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="P3" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
@@ -45851,7 +45861,7 @@
         <v>152</v>
       </c>
       <c r="F4" t="s">
-        <v>498</v>
+        <v>50</v>
       </c>
       <c r="G4" t="s">
         <v>278</v>
@@ -45863,10 +45873,10 @@
         <v>285</v>
       </c>
       <c r="O4" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="P4" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
@@ -45898,10 +45908,10 @@
         <v>7500</v>
       </c>
       <c r="O5" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="P5" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
@@ -45933,10 +45943,10 @@
         <v>5000</v>
       </c>
       <c r="O6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="P6" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
@@ -45962,16 +45972,16 @@
         <v>274</v>
       </c>
       <c r="H7" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="J7" t="s">
         <v>285</v>
       </c>
       <c r="O7" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="P7" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
@@ -45988,22 +45998,22 @@
         <v>27</v>
       </c>
       <c r="E8" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F8" t="s">
         <v>222</v>
       </c>
       <c r="G8" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="J8" t="s">
         <v>285</v>
       </c>
       <c r="O8" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="P8" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
@@ -46026,16 +46036,16 @@
         <v>222</v>
       </c>
       <c r="G9" t="s">
+        <v>509</v>
+      </c>
+      <c r="J9" t="s">
         <v>510</v>
       </c>
-      <c r="J9" t="s">
+      <c r="O9" t="s">
         <v>511</v>
       </c>
-      <c r="O9" t="s">
-        <v>512</v>
-      </c>
       <c r="P9" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
@@ -46070,7 +46080,7 @@
         <v>301</v>
       </c>
       <c r="P10" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
@@ -46105,7 +46115,7 @@
         <v>301</v>
       </c>
       <c r="P11" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
@@ -46134,7 +46144,7 @@
         <v>285</v>
       </c>
       <c r="P12" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
@@ -46151,7 +46161,7 @@
         <v>23</v>
       </c>
       <c r="E13" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F13" t="s">
         <v>49</v>
@@ -46166,10 +46176,81 @@
         <v>285</v>
       </c>
       <c r="P13" t="s">
-        <v>500</v>
+        <v>499</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2026</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>216</v>
+      </c>
+      <c r="D14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" t="s">
+        <v>129</v>
+      </c>
+      <c r="I14" t="s">
+        <v>262</v>
+      </c>
+      <c r="J14" t="s">
+        <v>84</v>
+      </c>
+      <c r="O14" t="s">
+        <v>513</v>
+      </c>
+      <c r="P14" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2026</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" t="s">
+        <v>216</v>
+      </c>
+      <c r="D15" t="s">
+        <v>262</v>
+      </c>
+      <c r="E15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" t="s">
+        <v>153</v>
+      </c>
+      <c r="G15" t="s">
+        <v>56</v>
+      </c>
+      <c r="I15" t="s">
+        <v>35</v>
+      </c>
+      <c r="J15" t="s">
+        <v>285</v>
+      </c>
+      <c r="O15" t="s">
+        <v>515</v>
+      </c>
+      <c r="P15" t="s">
+        <v>514</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
China Sprint and Quali
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2154" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D04F18B-2CA5-459A-BAAE-05B20E2FE5BC}"/>
+  <xr:revisionPtr revIDLastSave="2202" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10F42F54-033C-4D97-A892-AF87BEA1A9EC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10530" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10569" uniqueCount="519">
   <si>
     <t>Year</t>
   </si>
@@ -1577,6 +1577,12 @@
   </si>
   <si>
     <t>Verstappen said he was not impeded</t>
+  </si>
+  <si>
+    <t>Exceeding minimum time set by ECU behind SC</t>
+  </si>
+  <si>
+    <t>Isach Hadjar</t>
   </si>
 </sst>
 </file>
@@ -45721,7 +45727,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -46287,6 +46293,172 @@
         <v>514</v>
       </c>
     </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2026</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>216</v>
+      </c>
+      <c r="D17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17" t="s">
+        <v>45</v>
+      </c>
+      <c r="F17" t="s">
+        <v>153</v>
+      </c>
+      <c r="G17" t="s">
+        <v>271</v>
+      </c>
+      <c r="J17" t="s">
+        <v>11</v>
+      </c>
+      <c r="M17" t="s">
+        <v>245</v>
+      </c>
+      <c r="P17" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2026</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>216</v>
+      </c>
+      <c r="D18" t="s">
+        <v>262</v>
+      </c>
+      <c r="E18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" t="s">
+        <v>177</v>
+      </c>
+      <c r="G18" t="s">
+        <v>266</v>
+      </c>
+      <c r="I18" t="s">
+        <v>217</v>
+      </c>
+      <c r="J18" t="s">
+        <v>85</v>
+      </c>
+      <c r="K18">
+        <v>10</v>
+      </c>
+      <c r="P18" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2026</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>216</v>
+      </c>
+      <c r="D19" t="s">
+        <v>23</v>
+      </c>
+      <c r="E19" t="s">
+        <v>512</v>
+      </c>
+      <c r="F19" t="s">
+        <v>177</v>
+      </c>
+      <c r="G19" t="s">
+        <v>120</v>
+      </c>
+      <c r="J19" t="s">
+        <v>85</v>
+      </c>
+      <c r="K19">
+        <v>5</v>
+      </c>
+      <c r="O19" t="s">
+        <v>517</v>
+      </c>
+      <c r="P19" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2026</v>
+      </c>
+      <c r="B20">
+        <v>2</v>
+      </c>
+      <c r="C20" t="s">
+        <v>216</v>
+      </c>
+      <c r="D20" t="s">
+        <v>518</v>
+      </c>
+      <c r="E20" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" t="s">
+        <v>177</v>
+      </c>
+      <c r="G20" t="s">
+        <v>125</v>
+      </c>
+      <c r="J20" t="s">
+        <v>91</v>
+      </c>
+      <c r="P20" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2026</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>216</v>
+      </c>
+      <c r="D21" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" t="s">
+        <v>152</v>
+      </c>
+      <c r="F21" t="s">
+        <v>222</v>
+      </c>
+      <c r="G21" t="s">
+        <v>236</v>
+      </c>
+      <c r="J21" t="s">
+        <v>10</v>
+      </c>
+      <c r="L21">
+        <v>5000</v>
+      </c>
+      <c r="O21" t="s">
+        <v>139</v>
+      </c>
+      <c r="P21" t="s">
+        <v>514</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
China Q and R
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2203" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{835FD78A-A8E5-496C-9336-4F30A4917340}"/>
+  <xr:revisionPtr revIDLastSave="2221" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CCDFF87-94E6-4217-BF26-5AC80BEBEF29}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10569" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10585" uniqueCount="518">
   <si>
     <t>Year</t>
   </si>
@@ -45724,7 +45724,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -46456,6 +46456,73 @@
         <v>514</v>
       </c>
     </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2026</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>216</v>
+      </c>
+      <c r="D22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" t="s">
+        <v>45</v>
+      </c>
+      <c r="F22" t="s">
+        <v>48</v>
+      </c>
+      <c r="G22" t="s">
+        <v>271</v>
+      </c>
+      <c r="J22" t="s">
+        <v>11</v>
+      </c>
+      <c r="M22" t="s">
+        <v>245</v>
+      </c>
+      <c r="P22" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2026</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>216</v>
+      </c>
+      <c r="D23" t="s">
+        <v>30</v>
+      </c>
+      <c r="E23" t="s">
+        <v>39</v>
+      </c>
+      <c r="F23" t="s">
+        <v>49</v>
+      </c>
+      <c r="G23" t="s">
+        <v>266</v>
+      </c>
+      <c r="I23" t="s">
+        <v>218</v>
+      </c>
+      <c r="J23" t="s">
+        <v>85</v>
+      </c>
+      <c r="K23">
+        <v>10</v>
+      </c>
+      <c r="P23" t="s">
+        <v>514</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Japan FP1, FP2, FP3, Q
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2221" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8CCDFF87-94E6-4217-BF26-5AC80BEBEF29}"/>
+  <xr:revisionPtr revIDLastSave="2267" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92179759-0F4A-4339-9841-30DB0F480449}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10585" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10627" uniqueCount="521">
   <si>
     <t>Year</t>
   </si>
@@ -1580,6 +1580,15 @@
   </si>
   <si>
     <t>Exceeding minimum time set by ECU behind SC</t>
+  </si>
+  <si>
+    <t>Incident with Car 55</t>
+  </si>
+  <si>
+    <t>Gerd Ennser, Matthew Selley, Zhou Xiaoxu, Derek Warwick, Kazuhiro Tsuge</t>
+  </si>
+  <si>
+    <t>Neither driver to blame</t>
   </si>
 </sst>
 </file>
@@ -45724,7 +45733,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -46523,6 +46532,172 @@
         <v>514</v>
       </c>
     </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2026</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>173</v>
+      </c>
+      <c r="D24" t="s">
+        <v>197</v>
+      </c>
+      <c r="E24" t="s">
+        <v>265</v>
+      </c>
+      <c r="F24" t="s">
+        <v>52</v>
+      </c>
+      <c r="G24" t="s">
+        <v>203</v>
+      </c>
+      <c r="H24" t="s">
+        <v>518</v>
+      </c>
+      <c r="I24" t="s">
+        <v>111</v>
+      </c>
+      <c r="J24" t="s">
+        <v>285</v>
+      </c>
+      <c r="P24" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2026</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>173</v>
+      </c>
+      <c r="D25" t="s">
+        <v>36</v>
+      </c>
+      <c r="E25" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25" t="s">
+        <v>52</v>
+      </c>
+      <c r="G25" t="s">
+        <v>266</v>
+      </c>
+      <c r="I25" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" t="s">
+        <v>285</v>
+      </c>
+      <c r="O25" t="s">
+        <v>520</v>
+      </c>
+      <c r="P25" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2026</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+      <c r="C26" t="s">
+        <v>173</v>
+      </c>
+      <c r="D26" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" t="s">
+        <v>52</v>
+      </c>
+      <c r="G26" t="s">
+        <v>56</v>
+      </c>
+      <c r="I26" t="s">
+        <v>26</v>
+      </c>
+      <c r="J26" t="s">
+        <v>285</v>
+      </c>
+      <c r="P26" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2026</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>173</v>
+      </c>
+      <c r="D27" t="s">
+        <v>218</v>
+      </c>
+      <c r="E27" t="s">
+        <v>152</v>
+      </c>
+      <c r="F27" t="s">
+        <v>50</v>
+      </c>
+      <c r="G27" t="s">
+        <v>56</v>
+      </c>
+      <c r="I27" t="s">
+        <v>26</v>
+      </c>
+      <c r="J27" t="s">
+        <v>91</v>
+      </c>
+      <c r="P27" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>2026</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>173</v>
+      </c>
+      <c r="D28" t="s">
+        <v>195</v>
+      </c>
+      <c r="E28" t="s">
+        <v>42</v>
+      </c>
+      <c r="F28" t="s">
+        <v>51</v>
+      </c>
+      <c r="G28" t="s">
+        <v>56</v>
+      </c>
+      <c r="I28" t="s">
+        <v>27</v>
+      </c>
+      <c r="J28" t="s">
+        <v>91</v>
+      </c>
+      <c r="P28" t="s">
+        <v>519</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
I should've done this in the morning
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2296" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A6C41EC-C7AE-4386-9959-5200061F2AB3}"/>
+  <xr:revisionPtr revIDLastSave="2300" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40E97FAD-7719-43F2-9CFD-A0EDCE7B558E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46743,6 +46743,12 @@
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>2026</v>
+      </c>
+      <c r="B30">
+        <v>4</v>
+      </c>
       <c r="C30" t="s">
         <v>170</v>
       </c>
@@ -46772,6 +46778,12 @@
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>2026</v>
+      </c>
+      <c r="B31">
+        <v>4</v>
+      </c>
       <c r="C31" t="s">
         <v>170</v>
       </c>

</xml_diff>

<commit_message>
Miami S and Q
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2300" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40E97FAD-7719-43F2-9CFD-A0EDCE7B558E}"/>
+  <xr:revisionPtr revIDLastSave="2327" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{094DCA46-EF61-4C54-929A-326A69E0E6ED}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10650" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10675" uniqueCount="526">
   <si>
     <t>Year</t>
   </si>
@@ -1594,13 +1594,16 @@
     <t>Nish Shetty, Natalie Corsmit, Vitantonio Liuzzi, Steve Pence</t>
   </si>
   <si>
-    <t>Track Limits Violation</t>
-  </si>
-  <si>
     <t>Driver exceeded track limits in SQ1 and should have been eliminated, but was erroneously permitted to continue to SQ2</t>
   </si>
   <si>
     <t>Exceeded the 1:48.0 time limit between the Safety Car Lines</t>
+  </si>
+  <si>
+    <t>Team continued working on the car beyond covers-on time</t>
+  </si>
+  <si>
+    <t>Engine intake air pressure exceeded max. permitted limit</t>
   </si>
 </sst>
 </file>
@@ -45745,7 +45748,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -46762,7 +46765,7 @@
         <v>153</v>
       </c>
       <c r="G30" t="s">
-        <v>522</v>
+        <v>276</v>
       </c>
       <c r="J30" t="s">
         <v>11</v>
@@ -46771,7 +46774,7 @@
         <v>5</v>
       </c>
       <c r="O30" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="P30" t="s">
         <v>521</v>
@@ -46803,9 +46806,111 @@
         <v>285</v>
       </c>
       <c r="O31" t="s">
+        <v>523</v>
+      </c>
+      <c r="P31" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>2026</v>
+      </c>
+      <c r="B32">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" t="s">
+        <v>331</v>
+      </c>
+      <c r="E32" t="s">
+        <v>265</v>
+      </c>
+      <c r="F32" t="s">
+        <v>153</v>
+      </c>
+      <c r="G32" t="s">
+        <v>69</v>
+      </c>
+      <c r="J32" t="s">
+        <v>11</v>
+      </c>
+      <c r="M32" t="s">
+        <v>245</v>
+      </c>
+      <c r="O32" t="s">
         <v>524</v>
       </c>
-      <c r="P31" t="s">
+      <c r="P32" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>2026</v>
+      </c>
+      <c r="B33">
+        <v>4</v>
+      </c>
+      <c r="C33" t="s">
+        <v>170</v>
+      </c>
+      <c r="D33" t="s">
+        <v>262</v>
+      </c>
+      <c r="E33" t="s">
+        <v>38</v>
+      </c>
+      <c r="F33" t="s">
+        <v>177</v>
+      </c>
+      <c r="G33" t="s">
+        <v>127</v>
+      </c>
+      <c r="J33" t="s">
+        <v>85</v>
+      </c>
+      <c r="K33">
+        <v>5</v>
+      </c>
+      <c r="P33" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>2026</v>
+      </c>
+      <c r="B34">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>170</v>
+      </c>
+      <c r="D34" t="s">
+        <v>263</v>
+      </c>
+      <c r="E34" t="s">
+        <v>506</v>
+      </c>
+      <c r="F34" t="s">
+        <v>177</v>
+      </c>
+      <c r="G34" t="s">
+        <v>122</v>
+      </c>
+      <c r="H34" t="s">
+        <v>525</v>
+      </c>
+      <c r="J34" t="s">
+        <v>87</v>
+      </c>
+      <c r="O34" t="s">
+        <v>525</v>
+      </c>
+      <c r="P34" t="s">
         <v>521</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Canada sprint and quali
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2459" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7471DEC-47A0-46AF-917B-D38C6EF3FCAC}"/>
+  <xr:revisionPtr revIDLastSave="2560" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F742792A-5264-47E1-8B8A-19A712C44060}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10796" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10910" uniqueCount="544">
   <si>
     <t>Year</t>
   </si>
@@ -1640,6 +1640,24 @@
   </si>
   <si>
     <t>Exceeded time limit between the safety car lines</t>
+  </si>
+  <si>
+    <t>Failure to start formation lap</t>
+  </si>
+  <si>
+    <t>Procedural Infringement</t>
+  </si>
+  <si>
+    <t>Reported as having air released on the left rear tire with the wheel fitted to the car</t>
+  </si>
+  <si>
+    <t>Released into path of another car</t>
+  </si>
+  <si>
+    <t>Released from garage with wheel covers still fitted</t>
+  </si>
+  <si>
+    <t>Driver's first reprimand of the season</t>
   </si>
 </sst>
 </file>
@@ -45784,7 +45802,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P63"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -47445,6 +47463,472 @@
         <v>533</v>
       </c>
     </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>2026</v>
+      </c>
+      <c r="B50">
+        <v>5</v>
+      </c>
+      <c r="C50" t="s">
+        <v>168</v>
+      </c>
+      <c r="D50" t="s">
+        <v>463</v>
+      </c>
+      <c r="E50" t="s">
+        <v>509</v>
+      </c>
+      <c r="F50" t="s">
+        <v>150</v>
+      </c>
+      <c r="G50" t="s">
+        <v>268</v>
+      </c>
+      <c r="J50" t="s">
+        <v>11</v>
+      </c>
+      <c r="M50" t="s">
+        <v>242</v>
+      </c>
+      <c r="P50" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>2026</v>
+      </c>
+      <c r="B51">
+        <v>5</v>
+      </c>
+      <c r="C51" t="s">
+        <v>168</v>
+      </c>
+      <c r="D51" t="s">
+        <v>217</v>
+      </c>
+      <c r="E51" t="s">
+        <v>39</v>
+      </c>
+      <c r="F51" t="s">
+        <v>150</v>
+      </c>
+      <c r="G51" t="s">
+        <v>268</v>
+      </c>
+      <c r="J51" t="s">
+        <v>11</v>
+      </c>
+      <c r="M51" t="s">
+        <v>242</v>
+      </c>
+      <c r="P51" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>2026</v>
+      </c>
+      <c r="B52">
+        <v>5</v>
+      </c>
+      <c r="C52" t="s">
+        <v>168</v>
+      </c>
+      <c r="D52" t="s">
+        <v>25</v>
+      </c>
+      <c r="E52" t="s">
+        <v>149</v>
+      </c>
+      <c r="F52" t="s">
+        <v>150</v>
+      </c>
+      <c r="G52" t="s">
+        <v>268</v>
+      </c>
+      <c r="J52" t="s">
+        <v>11</v>
+      </c>
+      <c r="M52" t="s">
+        <v>242</v>
+      </c>
+      <c r="P52" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>2026</v>
+      </c>
+      <c r="B53">
+        <v>5</v>
+      </c>
+      <c r="C53" t="s">
+        <v>168</v>
+      </c>
+      <c r="D53" t="s">
+        <v>36</v>
+      </c>
+      <c r="E53" t="s">
+        <v>45</v>
+      </c>
+      <c r="F53" t="s">
+        <v>150</v>
+      </c>
+      <c r="G53" t="s">
+        <v>268</v>
+      </c>
+      <c r="J53" t="s">
+        <v>11</v>
+      </c>
+      <c r="M53" t="s">
+        <v>242</v>
+      </c>
+      <c r="P53" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>2026</v>
+      </c>
+      <c r="B54">
+        <v>5</v>
+      </c>
+      <c r="C54" t="s">
+        <v>168</v>
+      </c>
+      <c r="D54" t="s">
+        <v>28</v>
+      </c>
+      <c r="E54" t="s">
+        <v>147</v>
+      </c>
+      <c r="F54" t="s">
+        <v>174</v>
+      </c>
+      <c r="G54" t="s">
+        <v>504</v>
+      </c>
+      <c r="J54" t="s">
+        <v>282</v>
+      </c>
+      <c r="O54" t="s">
+        <v>538</v>
+      </c>
+      <c r="P54" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>2026</v>
+      </c>
+      <c r="B55">
+        <v>5</v>
+      </c>
+      <c r="C55" t="s">
+        <v>168</v>
+      </c>
+      <c r="D55" t="s">
+        <v>27</v>
+      </c>
+      <c r="E55" t="s">
+        <v>503</v>
+      </c>
+      <c r="F55" t="s">
+        <v>174</v>
+      </c>
+      <c r="G55" t="s">
+        <v>335</v>
+      </c>
+      <c r="I55" t="s">
+        <v>194</v>
+      </c>
+      <c r="J55" t="s">
+        <v>82</v>
+      </c>
+      <c r="K55">
+        <v>10</v>
+      </c>
+      <c r="P55" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>2026</v>
+      </c>
+      <c r="B56">
+        <v>5</v>
+      </c>
+      <c r="C56" t="s">
+        <v>168</v>
+      </c>
+      <c r="D56" t="s">
+        <v>23</v>
+      </c>
+      <c r="E56" t="s">
+        <v>509</v>
+      </c>
+      <c r="F56" t="s">
+        <v>174</v>
+      </c>
+      <c r="G56" t="s">
+        <v>65</v>
+      </c>
+      <c r="I56" t="s">
+        <v>194</v>
+      </c>
+      <c r="J56" t="s">
+        <v>82</v>
+      </c>
+      <c r="K56">
+        <v>10</v>
+      </c>
+      <c r="P56" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>2026</v>
+      </c>
+      <c r="B57">
+        <v>5</v>
+      </c>
+      <c r="C57" t="s">
+        <v>168</v>
+      </c>
+      <c r="D57" t="s">
+        <v>24</v>
+      </c>
+      <c r="E57" t="s">
+        <v>41</v>
+      </c>
+      <c r="F57" t="s">
+        <v>174</v>
+      </c>
+      <c r="G57" t="s">
+        <v>335</v>
+      </c>
+      <c r="I57" t="s">
+        <v>192</v>
+      </c>
+      <c r="J57" t="s">
+        <v>282</v>
+      </c>
+      <c r="P57" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>2026</v>
+      </c>
+      <c r="B58">
+        <v>5</v>
+      </c>
+      <c r="C58" t="s">
+        <v>168</v>
+      </c>
+      <c r="D58" t="s">
+        <v>30</v>
+      </c>
+      <c r="E58" t="s">
+        <v>39</v>
+      </c>
+      <c r="F58" t="s">
+        <v>174</v>
+      </c>
+      <c r="G58" t="s">
+        <v>119</v>
+      </c>
+      <c r="H58" t="s">
+        <v>539</v>
+      </c>
+      <c r="J58" t="s">
+        <v>282</v>
+      </c>
+      <c r="O58" t="s">
+        <v>540</v>
+      </c>
+      <c r="P58" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>2026</v>
+      </c>
+      <c r="B59">
+        <v>5</v>
+      </c>
+      <c r="C59" t="s">
+        <v>168</v>
+      </c>
+      <c r="D59" t="s">
+        <v>32</v>
+      </c>
+      <c r="E59" t="s">
+        <v>147</v>
+      </c>
+      <c r="F59" t="s">
+        <v>48</v>
+      </c>
+      <c r="G59" t="s">
+        <v>233</v>
+      </c>
+      <c r="I59" t="s">
+        <v>215</v>
+      </c>
+      <c r="J59" t="s">
+        <v>10</v>
+      </c>
+      <c r="L59">
+        <v>5000</v>
+      </c>
+      <c r="O59" t="s">
+        <v>541</v>
+      </c>
+      <c r="P59" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>2026</v>
+      </c>
+      <c r="B60">
+        <v>5</v>
+      </c>
+      <c r="C60" t="s">
+        <v>168</v>
+      </c>
+      <c r="D60" t="s">
+        <v>28</v>
+      </c>
+      <c r="E60" t="s">
+        <v>147</v>
+      </c>
+      <c r="F60" t="s">
+        <v>48</v>
+      </c>
+      <c r="G60" t="s">
+        <v>233</v>
+      </c>
+      <c r="J60" t="s">
+        <v>10</v>
+      </c>
+      <c r="L60">
+        <v>7000</v>
+      </c>
+      <c r="O60" t="s">
+        <v>542</v>
+      </c>
+      <c r="P60" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>2026</v>
+      </c>
+      <c r="B61">
+        <v>5</v>
+      </c>
+      <c r="C61" t="s">
+        <v>168</v>
+      </c>
+      <c r="D61" t="s">
+        <v>23</v>
+      </c>
+      <c r="E61" t="s">
+        <v>509</v>
+      </c>
+      <c r="F61" t="s">
+        <v>48</v>
+      </c>
+      <c r="G61" t="s">
+        <v>122</v>
+      </c>
+      <c r="J61" t="s">
+        <v>81</v>
+      </c>
+      <c r="O61" t="s">
+        <v>543</v>
+      </c>
+      <c r="P61" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>2026</v>
+      </c>
+      <c r="B62">
+        <v>5</v>
+      </c>
+      <c r="C62" t="s">
+        <v>168</v>
+      </c>
+      <c r="D62" t="s">
+        <v>24</v>
+      </c>
+      <c r="E62" t="s">
+        <v>41</v>
+      </c>
+      <c r="F62" t="s">
+        <v>48</v>
+      </c>
+      <c r="G62" t="s">
+        <v>53</v>
+      </c>
+      <c r="I62" t="s">
+        <v>25</v>
+      </c>
+      <c r="J62" t="s">
+        <v>282</v>
+      </c>
+      <c r="P62" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>2026</v>
+      </c>
+      <c r="B63">
+        <v>5</v>
+      </c>
+      <c r="C63" t="s">
+        <v>168</v>
+      </c>
+      <c r="D63" t="s">
+        <v>28</v>
+      </c>
+      <c r="E63" t="s">
+        <v>147</v>
+      </c>
+      <c r="F63" t="s">
+        <v>48</v>
+      </c>
+      <c r="G63" t="s">
+        <v>53</v>
+      </c>
+      <c r="I63" t="s">
+        <v>27</v>
+      </c>
+      <c r="J63" t="s">
+        <v>282</v>
+      </c>
+      <c r="P63" t="s">
+        <v>533</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Monaco FP1 and FP2
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2639" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0A13ABC-AB29-4AAE-BD4A-FF43F610198C}"/>
+  <xr:revisionPtr revIDLastSave="2707" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3110097F-C7E8-4C35-AE8B-E508E680DD99}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10987" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11049" uniqueCount="551">
   <si>
     <t>Year</t>
   </si>
@@ -1670,6 +1670,15 @@
   </si>
   <si>
     <t>Threw head restraint onto the track. Fine suspended for 12 month period</t>
+  </si>
+  <si>
+    <t>Driver was late to attend Thursday press conference</t>
+  </si>
+  <si>
+    <t>Fine suspended for period of 12 months</t>
+  </si>
+  <si>
+    <t>Garry Connelly, Derek Warwick, Tanja Geilhausen, Jean-Francois Calmes</t>
   </si>
 </sst>
 </file>
@@ -45814,7 +45823,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P73"/>
+  <dimension ref="A1:P81"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -48270,6 +48279,271 @@
         <v>533</v>
       </c>
     </row>
+    <row r="74" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>2026</v>
+      </c>
+      <c r="B74">
+        <v>6</v>
+      </c>
+      <c r="C74" t="s">
+        <v>138</v>
+      </c>
+      <c r="D74" t="s">
+        <v>35</v>
+      </c>
+      <c r="E74" t="s">
+        <v>42</v>
+      </c>
+      <c r="F74" t="s">
+        <v>175</v>
+      </c>
+      <c r="G74" t="s">
+        <v>199</v>
+      </c>
+      <c r="H74" t="s">
+        <v>548</v>
+      </c>
+      <c r="J74" t="s">
+        <v>10</v>
+      </c>
+      <c r="L74">
+        <v>5000</v>
+      </c>
+      <c r="O74" t="s">
+        <v>549</v>
+      </c>
+      <c r="P74" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>2026</v>
+      </c>
+      <c r="B75">
+        <v>6</v>
+      </c>
+      <c r="C75" t="s">
+        <v>138</v>
+      </c>
+      <c r="D75" t="s">
+        <v>29</v>
+      </c>
+      <c r="E75" t="s">
+        <v>41</v>
+      </c>
+      <c r="F75" t="s">
+        <v>175</v>
+      </c>
+      <c r="G75" t="s">
+        <v>199</v>
+      </c>
+      <c r="H75" t="s">
+        <v>548</v>
+      </c>
+      <c r="J75" t="s">
+        <v>10</v>
+      </c>
+      <c r="L75">
+        <v>5000</v>
+      </c>
+      <c r="O75" t="s">
+        <v>549</v>
+      </c>
+      <c r="P75" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>2026</v>
+      </c>
+      <c r="B76">
+        <v>6</v>
+      </c>
+      <c r="C76" t="s">
+        <v>138</v>
+      </c>
+      <c r="D76" t="s">
+        <v>37</v>
+      </c>
+      <c r="E76" t="s">
+        <v>38</v>
+      </c>
+      <c r="F76" t="s">
+        <v>530</v>
+      </c>
+      <c r="G76" t="s">
+        <v>270</v>
+      </c>
+      <c r="J76" t="s">
+        <v>10</v>
+      </c>
+      <c r="L76">
+        <v>100</v>
+      </c>
+      <c r="P76" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>2026</v>
+      </c>
+      <c r="B77">
+        <v>6</v>
+      </c>
+      <c r="C77" t="s">
+        <v>138</v>
+      </c>
+      <c r="D77" t="s">
+        <v>29</v>
+      </c>
+      <c r="E77" t="s">
+        <v>41</v>
+      </c>
+      <c r="F77" t="s">
+        <v>530</v>
+      </c>
+      <c r="G77" t="s">
+        <v>53</v>
+      </c>
+      <c r="I77" t="s">
+        <v>194</v>
+      </c>
+      <c r="J77" t="s">
+        <v>88</v>
+      </c>
+      <c r="P77" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>2026</v>
+      </c>
+      <c r="B78">
+        <v>6</v>
+      </c>
+      <c r="C78" t="s">
+        <v>138</v>
+      </c>
+      <c r="D78" t="s">
+        <v>328</v>
+      </c>
+      <c r="E78" t="s">
+        <v>262</v>
+      </c>
+      <c r="F78" t="s">
+        <v>530</v>
+      </c>
+      <c r="G78" t="s">
+        <v>53</v>
+      </c>
+      <c r="I78" t="s">
+        <v>192</v>
+      </c>
+      <c r="J78" t="s">
+        <v>88</v>
+      </c>
+      <c r="P78" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>2026</v>
+      </c>
+      <c r="B79">
+        <v>6</v>
+      </c>
+      <c r="C79" t="s">
+        <v>138</v>
+      </c>
+      <c r="D79" t="s">
+        <v>194</v>
+      </c>
+      <c r="E79" t="s">
+        <v>262</v>
+      </c>
+      <c r="F79" t="s">
+        <v>530</v>
+      </c>
+      <c r="G79" t="s">
+        <v>120</v>
+      </c>
+      <c r="J79" t="s">
+        <v>282</v>
+      </c>
+      <c r="P79" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>2026</v>
+      </c>
+      <c r="B80">
+        <v>6</v>
+      </c>
+      <c r="C80" t="s">
+        <v>138</v>
+      </c>
+      <c r="D80" t="s">
+        <v>32</v>
+      </c>
+      <c r="E80" t="s">
+        <v>147</v>
+      </c>
+      <c r="F80" t="s">
+        <v>531</v>
+      </c>
+      <c r="G80" t="s">
+        <v>270</v>
+      </c>
+      <c r="J80" t="s">
+        <v>10</v>
+      </c>
+      <c r="L80">
+        <v>100</v>
+      </c>
+      <c r="P80" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="81" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>2026</v>
+      </c>
+      <c r="B81">
+        <v>6</v>
+      </c>
+      <c r="C81" t="s">
+        <v>138</v>
+      </c>
+      <c r="D81" t="s">
+        <v>259</v>
+      </c>
+      <c r="E81" t="s">
+        <v>38</v>
+      </c>
+      <c r="F81" t="s">
+        <v>531</v>
+      </c>
+      <c r="G81" t="s">
+        <v>270</v>
+      </c>
+      <c r="J81" t="s">
+        <v>10</v>
+      </c>
+      <c r="L81">
+        <v>100</v>
+      </c>
+      <c r="P81" t="s">
+        <v>550</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Spain FP1, FP2, FP3
</commit_message>
<xml_diff>
--- a/data/F1Penalties.xlsx
+++ b/data/F1Penalties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce0ff7b57b908ca8/Desktop/F1 Notebooks/penaltyDashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2868" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0207AF6A-288E-49F7-AF59-F5F1D85081AE}"/>
+  <xr:revisionPtr revIDLastSave="2911" documentId="8_{37F5A6FD-68A1-49CA-8A46-44A4063429BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B47B7E5E-E7B3-45E4-B6CB-E975B70D75DA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11209" uniqueCount="558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11247" uniqueCount="564">
   <si>
     <t>Year</t>
   </si>
@@ -1700,6 +1700,24 @@
   </si>
   <si>
     <t>Applied after race</t>
+  </si>
+  <si>
+    <t>Overturned on Review</t>
+  </si>
+  <si>
+    <t>5 second time penalty overturned post race on review</t>
+  </si>
+  <si>
+    <t>Crossed the white line at pit exit</t>
+  </si>
+  <si>
+    <t>Felix Holter, Natalie Corsmit, Kipras Aleknavicius, Derek Warwick, David Domingo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fine </t>
+  </si>
+  <si>
+    <t>Drivers first reprimand of the season</t>
   </si>
 </sst>
 </file>
@@ -45844,7 +45862,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B3F-BE36-420E-A20B-01EC910651FC}">
-  <dimension ref="A1:P102"/>
+  <dimension ref="A1:P107"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="32.21875" customWidth="1"/>
@@ -48949,10 +48967,10 @@
         <v>270</v>
       </c>
       <c r="J93" t="s">
-        <v>82</v>
-      </c>
-      <c r="K93">
-        <v>5</v>
+        <v>558</v>
+      </c>
+      <c r="O93" t="s">
+        <v>559</v>
       </c>
       <c r="P93" t="s">
         <v>550</v>
@@ -49250,6 +49268,166 @@
       </c>
       <c r="P102" t="s">
         <v>550</v>
+      </c>
+    </row>
+    <row r="103" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A103">
+        <v>2026</v>
+      </c>
+      <c r="B103">
+        <v>7</v>
+      </c>
+      <c r="C103" t="s">
+        <v>96</v>
+      </c>
+      <c r="D103" t="s">
+        <v>32</v>
+      </c>
+      <c r="E103" t="s">
+        <v>147</v>
+      </c>
+      <c r="F103" t="s">
+        <v>531</v>
+      </c>
+      <c r="G103" t="s">
+        <v>120</v>
+      </c>
+      <c r="H103" t="s">
+        <v>560</v>
+      </c>
+      <c r="J103" t="s">
+        <v>88</v>
+      </c>
+      <c r="P103" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="104" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A104">
+        <v>2026</v>
+      </c>
+      <c r="B104">
+        <v>7</v>
+      </c>
+      <c r="C104" t="s">
+        <v>96</v>
+      </c>
+      <c r="D104" t="s">
+        <v>463</v>
+      </c>
+      <c r="E104" t="s">
+        <v>509</v>
+      </c>
+      <c r="F104" t="s">
+        <v>531</v>
+      </c>
+      <c r="G104" t="s">
+        <v>270</v>
+      </c>
+      <c r="J104" t="s">
+        <v>10</v>
+      </c>
+      <c r="L104">
+        <v>100</v>
+      </c>
+      <c r="P104" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="105" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A105">
+        <v>2026</v>
+      </c>
+      <c r="B105">
+        <v>7</v>
+      </c>
+      <c r="C105" t="s">
+        <v>96</v>
+      </c>
+      <c r="D105" t="s">
+        <v>23</v>
+      </c>
+      <c r="E105" t="s">
+        <v>509</v>
+      </c>
+      <c r="F105" t="s">
+        <v>531</v>
+      </c>
+      <c r="G105" t="s">
+        <v>270</v>
+      </c>
+      <c r="J105" t="s">
+        <v>562</v>
+      </c>
+      <c r="L105">
+        <v>500</v>
+      </c>
+      <c r="P105" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="106" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A106">
+        <v>2026</v>
+      </c>
+      <c r="B106">
+        <v>7</v>
+      </c>
+      <c r="C106" t="s">
+        <v>96</v>
+      </c>
+      <c r="D106" t="s">
+        <v>28</v>
+      </c>
+      <c r="E106" t="s">
+        <v>147</v>
+      </c>
+      <c r="F106" t="s">
+        <v>532</v>
+      </c>
+      <c r="G106" t="s">
+        <v>270</v>
+      </c>
+      <c r="J106" t="s">
+        <v>10</v>
+      </c>
+      <c r="L106">
+        <v>600</v>
+      </c>
+      <c r="P106" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="107" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A107">
+        <v>2026</v>
+      </c>
+      <c r="B107">
+        <v>7</v>
+      </c>
+      <c r="C107" t="s">
+        <v>96</v>
+      </c>
+      <c r="D107" t="s">
+        <v>259</v>
+      </c>
+      <c r="E107" t="s">
+        <v>38</v>
+      </c>
+      <c r="F107" t="s">
+        <v>532</v>
+      </c>
+      <c r="G107" t="s">
+        <v>264</v>
+      </c>
+      <c r="J107" t="s">
+        <v>81</v>
+      </c>
+      <c r="O107" t="s">
+        <v>563</v>
+      </c>
+      <c r="P107" t="s">
+        <v>561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>